<commit_message>
feat: support imported filename without parenthesis
</commit_message>
<xml_diff>
--- a/static/Class IX (2024).xlsx
+++ b/static/Class IX (2024).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026 Projects\My-Darpan\Darpan-mobile\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3EB639-F9B2-45E1-BD1A-B33B7F86A76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8D6C02-E7ED-4B8F-97D7-FF5EB88CAC9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7005" yWindow="1020" windowWidth="14640" windowHeight="14580" xr2:uid="{96A36A53-D1E9-448B-B448-63641815E4B3}"/>
+    <workbookView xWindow="2550" yWindow="615" windowWidth="14640" windowHeight="14580" xr2:uid="{96A36A53-D1E9-448B-B448-63641815E4B3}"/>
   </bookViews>
   <sheets>
     <sheet name="B1" sheetId="2" r:id="rId1"/>

</xml_diff>